<commit_message>
Phase 3 Step B: segment, classify and file documents with audited unmasked originals (A35)
Deterministic signature library, bundle segmentation, classifier fallback,
party and period assignment, A32 supersession with undo, durable steps and
the intake, documents and filing review screens.

Record owner ruling A35: derived and stored data stay masked; originals open
unmasked for admin and operator roles only, one audit event per open, signed
no-store links, and startup refuses REAL_DATA_MODE with PUBLIC_DEMO_MODE.
Tests cover A35 conditions 1, 2 and 4; the review screen shows the notice.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/deals/deal-a/incoming/batch-1/Seller/Fwd - closing docs/fin-2025.XLSX
+++ b/fixtures/deals/deal-a/incoming/batch-1/Seller/Fwd - closing docs/fin-2025.XLSX
@@ -398,104 +398,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
-  <cols>
-    <col min="1" max="1" width="120.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>SYNTHETIC</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Income Statement</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>SYNTHETIC</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Year-end Income Statement and Balance Sheet</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Simplified training facsimile - never submit to an agency or lender</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Name: Varnholt Climate Services LLC</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Period: 2025</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Record: fin-2025</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Address: 14 Velnoric Way, Tazmervale, ZZ 00000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Contact: fixture@example.com | (202) 555-0142</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>revenue: 1484000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>net income: 140000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Signature: e-signed; Date: 2026-08-31</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Electronic signature envelope: SYNTHETIC-deal-a-fin-2025</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Signer: Varnholt Climate Services LLC</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Prepared from synthetic documents. For lender review only.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>SYNTHETIC - For lender review only</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B17"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
@@ -507,7 +409,7 @@
         <v>SYNTHETIC</v>
       </c>
       <c r="B1" t="str">
-        <v>Balance Sheet</v>
+        <v>Income Statement</v>
       </c>
     </row>
     <row r="2">
@@ -542,42 +444,42 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Address: 14 Velnoric Way, Tazmervale, ZZ 00000</v>
+        <v>Document date: 2026-08-31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Contact: fixture@example.com | (202) 555-0142</v>
+        <v>Address: 14 Velnoric Way, Tazmervale, ZZ 00000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>total assets: 500000</v>
+        <v>Contact: fixture@example.com | (202) 555-0142</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>total liabilities: 100000</v>
+        <v>revenue: 1484000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Signature: e-signed; Date: 2026-08-31</v>
+        <v>net income: 140000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Electronic signature envelope: SYNTHETIC-deal-a-fin-2025</v>
+        <v>Signature: e-signed; Date: 2026-08-31</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Signer: Varnholt Climate Services LLC</v>
+        <v>Electronic signature envelope: SYNTHETIC-deal-a-fin-2025</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Equity: 400000</v>
+        <v>Signer: Varnholt Climate Services LLC</v>
       </c>
     </row>
     <row r="16">
@@ -595,4 +497,112 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="120.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SYNTHETIC</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Balance Sheet</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SYNTHETIC</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Year-end Income Statement and Balance Sheet</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Simplified training facsimile - never submit to an agency or lender</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Name: Varnholt Climate Services LLC</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Period: 2025</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Record: fin-2025</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Document date: 2026-08-31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Address: 14 Velnoric Way, Tazmervale, ZZ 00000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Contact: fixture@example.com | (202) 555-0142</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>total assets: 500000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>total liabilities: 100000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Signature: e-signed; Date: 2026-08-31</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Electronic signature envelope: SYNTHETIC-deal-a-fin-2025</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Signer: Varnholt Climate Services LLC</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Equity: 400000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Prepared from synthetic documents. For lender review only.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>SYNTHETIC - For lender review only</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>